<commit_message>
ya empecé con redes neuronales
</commit_message>
<xml_diff>
--- a/5_svm/2_datos/1_raw/1_80_20/3_meteo_epi_2021-2026_1_rezagos_meteo_test_80_20.xlsx
+++ b/5_svm/2_datos/1_raw/1_80_20/3_meteo_epi_2021-2026_1_rezagos_meteo_test_80_20.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -501,7 +501,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -534,7 +534,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>

</xml_diff>